<commit_message>
+ Add Armor 07 - 08 and fix bug about passive.
</commit_message>
<xml_diff>
--- a/Tool/data/Shop.xlsx
+++ b/Tool/data/Shop.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -15,12 +15,12 @@
     <sheet name="ShopProducts" sheetId="1" r:id="rId1"/>
     <sheet name="BundleContents" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="102">
   <si>
     <t>ProductID</t>
   </si>
@@ -70,45 +70,126 @@
     <t>SHOP_RARE_01</t>
   </si>
   <si>
+    <t>RareLimit</t>
+  </si>
+  <si>
+    <t>JadeShop</t>
+  </si>
+  <si>
+    <t>SingleItem</t>
+  </si>
+  <si>
+    <t>SunWukong</t>
+  </si>
+  <si>
+    <t>Jade</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
     <t>SHOP_RARE_02</t>
   </si>
   <si>
+    <t>Armor01_Belt</t>
+  </si>
+  <si>
+    <t>Lifetime</t>
+  </si>
+  <si>
     <t>SHOP_RARE_03</t>
   </si>
   <si>
+    <t>TangSanZang</t>
+  </si>
+  <si>
     <t>SHOP_RARE_04</t>
   </si>
   <si>
+    <t>common_exp</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
     <t>SHOP_RARE_05</t>
   </si>
   <si>
+    <t>Fried_Radish_Balls</t>
+  </si>
+  <si>
     <t>SHOP_RARE_06</t>
   </si>
   <si>
+    <t>Dragon_Bread_Noodies</t>
+  </si>
+  <si>
     <t>SHOP_RARE_07</t>
   </si>
   <si>
+    <t>CoinShop</t>
+  </si>
+  <si>
+    <t>Murshroom_Steamed_Buns</t>
+  </si>
+  <si>
+    <t>Coin</t>
+  </si>
+  <si>
     <t>SHOP_RARE_08</t>
   </si>
   <si>
+    <t>Tofu_Soup</t>
+  </si>
+  <si>
     <t>SHOP_RARE_09</t>
   </si>
   <si>
+    <t>Lamian_Noodies</t>
+  </si>
+  <si>
     <t>SHOP_RARE_10</t>
   </si>
   <si>
+    <t>fine_exp</t>
+  </si>
+  <si>
     <t>SHOP_RARE_11</t>
   </si>
   <si>
+    <t>rare_exp</t>
+  </si>
+  <si>
     <t>SHOP_RARE_12</t>
   </si>
   <si>
+    <t>ZhuBaJie</t>
+  </si>
+  <si>
     <t>SHOP_TIME_01</t>
   </si>
   <si>
+    <t>TimeSale</t>
+  </si>
+  <si>
+    <t>supreme_exp</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-30</t>
+  </si>
+  <si>
     <t>SHOP_TIME_02</t>
   </si>
   <si>
+    <t>Garnet_Gemstone</t>
+  </si>
+  <si>
     <t>SHOP_TIME_03</t>
   </si>
   <si>
@@ -118,115 +199,70 @@
     <t>SHOP_COMBO_01</t>
   </si>
   <si>
+    <t>ComboPack</t>
+  </si>
+  <si>
+    <t>Bundle</t>
+  </si>
+  <si>
+    <t>BUNDLE_JADE_01</t>
+  </si>
+  <si>
     <t>SHOP_COMBO_02</t>
   </si>
   <si>
+    <t>BUNDLE_JADE_02</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
     <t>SHOP_COMBO_03</t>
   </si>
   <si>
+    <t>BUNDLE_COIN_01</t>
+  </si>
+  <si>
     <t>SHOP_COMBO_04</t>
   </si>
   <si>
-    <t>RareLimit</t>
-  </si>
-  <si>
-    <t>TimeSale</t>
-  </si>
-  <si>
-    <t>ComboPack</t>
-  </si>
-  <si>
-    <t>JadeShop</t>
-  </si>
-  <si>
-    <t>CoinShop</t>
-  </si>
-  <si>
-    <t>SingleItem</t>
-  </si>
-  <si>
-    <t>Bundle</t>
-  </si>
-  <si>
-    <t>SunWukong</t>
-  </si>
-  <si>
-    <t>Armor01_Belt</t>
-  </si>
-  <si>
-    <t>TangSanZang</t>
-  </si>
-  <si>
-    <t>common_exp</t>
-  </si>
-  <si>
-    <t>Fried_Radish_Balls</t>
-  </si>
-  <si>
-    <t>Dragon_Bread_Noodies</t>
-  </si>
-  <si>
-    <t>Murshroom_Steamed_Buns</t>
-  </si>
-  <si>
-    <t>Tofu_Soup</t>
-  </si>
-  <si>
-    <t>Lamian_Noodies</t>
-  </si>
-  <si>
-    <t>fine_exp</t>
-  </si>
-  <si>
-    <t>rare_exp</t>
-  </si>
-  <si>
-    <t>ZhuBaJie</t>
-  </si>
-  <si>
-    <t>supreme_exp</t>
-  </si>
-  <si>
-    <t>Garnet_Gemstone</t>
-  </si>
-  <si>
-    <t>BUNDLE_JADE_01</t>
-  </si>
-  <si>
-    <t>BUNDLE_JADE_02</t>
-  </si>
-  <si>
-    <t>BUNDLE_COIN_01</t>
-  </si>
-  <si>
     <t>BUNDLE_COIN_02</t>
   </si>
   <si>
-    <t>Jade</t>
-  </si>
-  <si>
-    <t>Coin</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>Lifetime</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>2026-05-01</t>
-  </si>
-  <si>
-    <t>2026-05-30</t>
+    <t>SHOP_ARMOR_01_A</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR01_01</t>
+  </si>
+  <si>
+    <t>SHOP_ARMOR_01_B</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR01_02</t>
+  </si>
+  <si>
+    <t>SHOP_ARMOR_07_A</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR07_01</t>
+  </si>
+  <si>
+    <t>SHOP_ARMOR_07_B</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR07_02</t>
+  </si>
+  <si>
+    <t>SHOP_ARMOR_08_A</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR08_01</t>
+  </si>
+  <si>
+    <t>SHOP_ARMOR_08_B</t>
+  </si>
+  <si>
+    <t>BUNDLE_ARMOR08_02</t>
   </si>
   <si>
     <t>BundleID</t>
@@ -239,13 +275,64 @@
   </si>
   <si>
     <t>Nimbus_Cudgel</t>
+  </si>
+  <si>
+    <t>Armor01_Helmet</t>
+  </si>
+  <si>
+    <t>Armor01_Chestplate</t>
+  </si>
+  <si>
+    <t>Armor01_Gloves</t>
+  </si>
+  <si>
+    <t>Armor01_Boots</t>
+  </si>
+  <si>
+    <t>Armor01_Ring</t>
+  </si>
+  <si>
+    <t>Armor07_Helmet</t>
+  </si>
+  <si>
+    <t>Armor07_Chestplate</t>
+  </si>
+  <si>
+    <t>Armor07_Gloves</t>
+  </si>
+  <si>
+    <t>Armor07_Boots</t>
+  </si>
+  <si>
+    <t>Armor07_Belt</t>
+  </si>
+  <si>
+    <t>Armor07_Ring</t>
+  </si>
+  <si>
+    <t>Armor08_Helmet</t>
+  </si>
+  <si>
+    <t>Armor08_Chestplate</t>
+  </si>
+  <si>
+    <t>Armor08_Gloves</t>
+  </si>
+  <si>
+    <t>Armor08_Boots</t>
+  </si>
+  <si>
+    <t>Armor08_Belt</t>
+  </si>
+  <si>
+    <t>Armor08_Ring</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,24 +340,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -278,29 +363,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -606,8 +682,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -661,843 +751,1089 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H2">
+        <v>19</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="2">
         <v>100</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="2">
         <v>150</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="2">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3">
+        <v>23</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2">
         <v>500</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="2">
         <v>0</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>60</v>
-      </c>
-      <c r="H4">
+        <v>26</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2">
         <v>10000</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="2">
         <v>12000</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>5</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
       <c r="E5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>60</v>
-      </c>
-      <c r="H5">
+        <v>28</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2">
         <v>5000</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="2">
         <v>0</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>5</v>
       </c>
       <c r="K5" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6">
+        <v>31</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2">
         <v>1000</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="2">
         <v>12000</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>5</v>
       </c>
       <c r="K6" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H7">
+      <c r="H7" s="2">
         <v>1200</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="2">
         <v>0</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <v>5</v>
       </c>
       <c r="K7" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" s="2">
+        <v>100</v>
+      </c>
+      <c r="I8" s="2">
+        <v>150</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1</v>
+      </c>
+      <c r="K8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8" t="s">
-        <v>61</v>
-      </c>
-      <c r="H8">
-        <v>100</v>
-      </c>
-      <c r="I8">
-        <v>150</v>
-      </c>
-      <c r="J8">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
-        <v>62</v>
-      </c>
       <c r="N8" t="b">
         <v>1</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
         <v>35</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
         <v>39</v>
       </c>
-      <c r="D9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9" t="s">
-        <v>61</v>
-      </c>
-      <c r="H9">
+      <c r="F9" s="3">
+        <v>1</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" s="2">
         <v>500</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="2">
         <v>0</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="2">
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
         <v>35</v>
       </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10">
+        <v>41</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" s="2">
         <v>10000</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="2">
         <v>12000</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="2">
         <v>5</v>
       </c>
       <c r="K10" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
         <v>35</v>
       </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11">
+        <v>43</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="2">
         <v>5000</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="2">
         <v>0</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="2">
         <v>5</v>
       </c>
       <c r="K11" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>35</v>
       </c>
-      <c r="C12" t="s">
-        <v>39</v>
-      </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="2">
         <v>1000</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="2">
         <v>12000</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="2">
         <v>5</v>
       </c>
       <c r="K12" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
-        <v>39</v>
-      </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13">
+        <v>47</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="2">
         <v>1200</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="2">
         <v>0</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="2">
         <v>5</v>
       </c>
       <c r="K13" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14">
+        <v>50</v>
+      </c>
+      <c r="F14" s="3">
         <v>10</v>
       </c>
-      <c r="G14" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14">
+      <c r="G14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" s="2">
         <v>50</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="2">
         <v>100</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="2">
         <v>5</v>
       </c>
       <c r="K14" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L14" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="M14" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
         <v>55</v>
       </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15">
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="2">
         <v>80</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="2">
         <v>120</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="2">
         <v>5</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L15" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="M15" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="3">
+        <v>10</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I16" s="2">
+        <v>8000</v>
+      </c>
+      <c r="J16" s="2">
+        <v>5</v>
+      </c>
+      <c r="K16" t="s">
         <v>51</v>
       </c>
-      <c r="F16">
-        <v>10</v>
-      </c>
-      <c r="G16" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16">
-        <v>5000</v>
-      </c>
-      <c r="I16">
-        <v>8000</v>
-      </c>
-      <c r="J16">
-        <v>5</v>
-      </c>
-      <c r="K16" t="s">
-        <v>65</v>
-      </c>
       <c r="L16" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="M16" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
-      </c>
-      <c r="F17">
+        <v>41</v>
+      </c>
+      <c r="F17" s="3">
         <v>5</v>
       </c>
-      <c r="G17" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17">
+      <c r="G17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="2">
         <v>8000</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="2">
         <v>10000</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="2">
         <v>5</v>
       </c>
       <c r="K17" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L17" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="M17" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18">
+        <v>61</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H18" s="2">
         <v>300</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="2">
         <v>500</v>
       </c>
-      <c r="J18">
-        <v>1</v>
+      <c r="J18" s="2">
+        <v>10</v>
       </c>
       <c r="K18" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
-      </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
-      <c r="G19" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19">
+        <v>63</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" s="2">
         <v>600</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="2">
         <v>800</v>
       </c>
-      <c r="J19">
-        <v>1</v>
+      <c r="J19" s="2">
+        <v>10</v>
       </c>
       <c r="K19" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C20" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" t="s">
-        <v>41</v>
-      </c>
-      <c r="E20" t="s">
-        <v>58</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20">
+      <c r="H20" s="2">
         <v>20000</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="2">
         <v>30000</v>
       </c>
-      <c r="J20">
-        <v>1</v>
+      <c r="J20" s="2">
+        <v>10</v>
       </c>
       <c r="K20" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" t="s">
-        <v>41</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="H21" s="2">
+        <v>50000</v>
+      </c>
+      <c r="I21" s="2">
+        <v>70000</v>
+      </c>
+      <c r="J21" s="2">
+        <v>10</v>
+      </c>
+      <c r="K21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B22" t="s">
         <v>59</v>
       </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H21">
-        <v>50000</v>
-      </c>
-      <c r="I21">
-        <v>70000</v>
-      </c>
-      <c r="J21">
-        <v>1</v>
-      </c>
-      <c r="K21" t="s">
-        <v>66</v>
-      </c>
-      <c r="N21" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21">
+      <c r="C22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H22" s="2">
+        <v>800</v>
+      </c>
+      <c r="I22" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J22" s="2">
+        <v>10</v>
+      </c>
+      <c r="K22" t="s">
+        <v>29</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" s="2">
+        <v>800</v>
+      </c>
+      <c r="I23" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J23" s="2">
+        <v>10</v>
+      </c>
+      <c r="K23" t="s">
+        <v>29</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="3">
+        <v>1</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H24" s="2">
+        <v>800</v>
+      </c>
+      <c r="I24" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J24" s="2">
+        <v>10</v>
+      </c>
+      <c r="K24" t="s">
+        <v>29</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>75</v>
+      </c>
+      <c r="B25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" s="2">
+        <v>800</v>
+      </c>
+      <c r="I25" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J25" s="2">
+        <v>10</v>
+      </c>
+      <c r="K25" t="s">
+        <v>29</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25" s="2">
         <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" t="s">
+        <v>78</v>
+      </c>
+      <c r="F26" s="3">
+        <v>1</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="2">
+        <v>800</v>
+      </c>
+      <c r="I26" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J26" s="2">
+        <v>10</v>
+      </c>
+      <c r="K26" t="s">
+        <v>29</v>
+      </c>
+      <c r="N26" t="b">
+        <v>1</v>
+      </c>
+      <c r="O26" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" t="s">
+        <v>80</v>
+      </c>
+      <c r="F27" s="3">
+        <v>1</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2">
+        <v>800</v>
+      </c>
+      <c r="I27" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J27" s="2">
+        <v>10</v>
+      </c>
+      <c r="K27" t="s">
+        <v>29</v>
+      </c>
+      <c r="N27" t="b">
+        <v>1</v>
+      </c>
+      <c r="O27" s="2">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1507,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
@@ -1515,22 +1851,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>71</v>
+      <c r="A1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -1538,10 +1874,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1549,10 +1885,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1560,7 +1896,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
         <v>55</v>
@@ -1571,10 +1907,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1582,7 +1918,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
         <v>55</v>
@@ -1593,10 +1929,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C8">
         <v>10</v>
@@ -1604,10 +1940,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -1615,10 +1951,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C10">
         <v>20</v>
@@ -1626,10 +1962,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -1637,10 +1973,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1648,10 +1984,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C13">
         <v>10</v>
@@ -1659,10 +1995,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C14">
         <v>50</v>
@@ -1670,13 +2006,211 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C15">
         <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" t="s">
+        <v>96</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Fix bug stuck game after fish battle in Main Quest.
</commit_message>
<xml_diff>
--- a/Tool/data/Shop.xlsx
+++ b/Tool/data/Shop.xlsx
@@ -5131,7 +5131,7 @@
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5162,7 +5162,7 @@
         <v>20</v>
       </c>
       <c r="D2">
-        <v>1000000</v>
+        <v>10000000</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
+ Add exp redeem code reward.
</commit_message>
<xml_diff>
--- a/Tool/data/Shop.xlsx
+++ b/Tool/data/Shop.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityUdeme\Trunk_Android\MyTemplateAndroid\MyTemplate_Android\Tool\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityUdeme\MyTemplate\MyTemplate\Tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -17,12 +17,12 @@
     <sheet name="SevenDayLogin" sheetId="3" r:id="rId3"/>
     <sheet name="RedeemCode" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="237">
   <si>
     <t>ProductID</t>
   </si>
@@ -730,6 +730,9 @@
   </si>
   <si>
     <t>`</t>
+  </si>
+  <si>
+    <t>GIFT_EXP</t>
   </si>
 </sst>
 </file>
@@ -5129,7 +5132,7 @@
   <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
     <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -5155,7 +5158,7 @@
       <c r="A2" t="s">
         <v>230</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C2" t="s">
@@ -5172,7 +5175,7 @@
       <c r="A3" t="s">
         <v>231</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C3" t="s">
@@ -5189,7 +5192,7 @@
       <c r="A4" t="s">
         <v>232</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C4" t="s">
@@ -5206,7 +5209,7 @@
       <c r="A5" t="s">
         <v>233</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C5" t="s">
@@ -5223,7 +5226,7 @@
       <c r="A6" t="s">
         <v>234</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C6" t="s">
@@ -5233,6 +5236,23 @@
         <v>100</v>
       </c>
       <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>